<commit_message>
Correct five points in Resampling and Simulation
The median has no simple standard-error formula, but it does have an exact order-statistic interval, and the notebook now prints it ($100,700 to $111,100) beside the bootstrap's. The bootstrap needs independent, representative data and fails for the maximum, and BCa matches the percentile interval here because its correction terms come out near zero. The scipy call takes (data,), and the salaries are a realistic teaching dataset.
</commit_message>
<xml_diff>
--- a/data/resampling-and-simulation--salaries.xlsx
+++ b/data/resampling-and-simulation--salaries.xlsx
@@ -6015,14 +6015,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WHAT IS CAPTURED: an HR compensation export.</t>
+          <t>WHAT IS CAPTURED: an HR compensation export (a realistic teaching dataset written for the book).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Goal: a confidence interval for the MEDIAN salary - there is no simple formula, so we BOOTSTRAP.</t>
+          <t>Goal: a confidence interval for the MEDIAN salary. It has no simple standard-error formula, so we BOOTSTRAP (and compare the exact order-statistic interval).</t>
         </is>
       </c>
     </row>

</xml_diff>